<commit_message>
Fixed local replica, missing pulse shaping optimisation
</commit_message>
<xml_diff>
--- a/Algorithm/Acquisition/SignalCharacteristics/signalData.xlsx
+++ b/Algorithm/Acquisition/SignalCharacteristics/signalData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cranfield-my.sharepoint.com/personal/a_lavinorejas_261_cranfield_ac_uk/Documents/Documents/Group Design Project/Cranfield-LEO-PNT/Algorithm/Acquisition/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cranfield-my.sharepoint.com/personal/a_lavinorejas_261_cranfield_ac_uk/Documents/Documents/Group Design Project/Cranfield-LEO-PNT/Algorithm/Acquisition/SignalCharacteristics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="8_{31AC4230-72C4-4582-8E31-DEF67DFFC137}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{472921F9-5837-43F7-A322-0337B65D3855}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="8_{31AC4230-72C4-4582-8E31-DEF67DFFC137}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C251215-0BE3-45E3-A109-4D1766DBCABA}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="1100" windowWidth="19200" windowHeight="9980" xr2:uid="{C1A3185A-F3C0-4606-B2D6-D4D09FADDBA2}"/>
+    <workbookView xWindow="-27150" yWindow="12240" windowWidth="21600" windowHeight="10980" xr2:uid="{C1A3185A-F3C0-4606-B2D6-D4D09FADDBA2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>ID</t>
   </si>
@@ -66,6 +66,9 @@
   </si>
   <si>
     <t>SymbolFreq</t>
+  </si>
+  <si>
+    <t>OW_BladeRF_20dBatt_6GB.bin</t>
   </si>
 </sst>
 </file>
@@ -446,7 +449,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C04845A8-D2B3-4AA5-B1E2-4210EB6AE0BD}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -504,7 +507,7 @@
         <v>320000000</v>
       </c>
       <c r="D3">
-        <f t="shared" ref="D3:D4" si="0">230400000</f>
+        <f t="shared" ref="D3:D5" si="0">230400000</f>
         <v>230400000</v>
       </c>
       <c r="E3" t="s">
@@ -523,6 +526,22 @@
         <v>360000000</v>
       </c>
       <c r="D4">
+        <f t="shared" si="0"/>
+        <v>230400000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.5">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5">
+        <f>60000000</f>
+        <v>60000000</v>
+      </c>
+      <c r="D5">
         <f t="shared" si="0"/>
         <v>230400000</v>
       </c>

</xml_diff>

<commit_message>
Added signal to spreadsheet and update peaksCorrelation
</commit_message>
<xml_diff>
--- a/Algorithm/Acquisition/SignalCharacteristics/signalData.xlsx
+++ b/Algorithm/Acquisition/SignalCharacteristics/signalData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cranfield-my.sharepoint.com/personal/a_lavinorejas_261_cranfield_ac_uk/Documents/Documents/Group Design Project/Cranfield-LEO-PNT/Algorithm/Acquisition/SignalCharacteristics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="8_{31AC4230-72C4-4582-8E31-DEF67DFFC137}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C251215-0BE3-45E3-A109-4D1766DBCABA}"/>
+  <xr:revisionPtr revIDLastSave="39" documentId="8_{31AC4230-72C4-4582-8E31-DEF67DFFC137}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37EBFB50-868C-4B66-B742-44A8AA5E3B44}"/>
   <bookViews>
-    <workbookView xWindow="-27150" yWindow="12240" windowWidth="21600" windowHeight="10980" xr2:uid="{C1A3185A-F3C0-4606-B2D6-D4D09FADDBA2}"/>
+    <workbookView xWindow="747" yWindow="993" windowWidth="19200" windowHeight="9980" xr2:uid="{C1A3185A-F3C0-4606-B2D6-D4D09FADDBA2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>ID</t>
   </si>
@@ -68,7 +68,13 @@
     <t>SymbolFreq</t>
   </si>
   <si>
-    <t>OW_BladeRF_20dBatt_6GB.bin</t>
+    <t>LNB_BladeRF_5s.bin</t>
+  </si>
+  <si>
+    <t>OW_BladeRF_6GB_real.bin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BladeRF generated signal, limitation on Sampling frequency </t>
   </si>
 </sst>
 </file>
@@ -449,7 +455,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C04845A8-D2B3-4AA5-B1E2-4210EB6AE0BD}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -507,7 +513,7 @@
         <v>320000000</v>
       </c>
       <c r="D3">
-        <f t="shared" ref="D3:D5" si="0">230400000</f>
+        <f t="shared" ref="D3:D6" si="0">230400000</f>
         <v>230400000</v>
       </c>
       <c r="E3" t="s">
@@ -535,13 +541,32 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C5">
         <f>60000000</f>
         <v>60000000</v>
       </c>
       <c r="D5">
+        <f t="shared" si="0"/>
+        <v>230400000</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.5">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6">
+        <f>60000000</f>
+        <v>60000000</v>
+      </c>
+      <c r="D6">
         <f t="shared" si="0"/>
         <v>230400000</v>
       </c>

</xml_diff>